<commit_message>
Respaldo automático: 2026-10-14 09:33
</commit_message>
<xml_diff>
--- a/2026-2/AsistenciaFPE-1.xlsx
+++ b/2026-2/AsistenciaFPE-1.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unicordoba/Documents/Cursos/FPEI/2026-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B478C7-A4A9-0745-BFE3-D76470B3C9E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE37022-042E-BB4A-B016-818BC2258F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -825,47 +838,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="21.5" customWidth="1"/>
-    <col min="4" max="8" width="24.5" customWidth="1"/>
+    <col min="2" max="4" width="21.5" customWidth="1"/>
+    <col min="5" max="9" width="24.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -873,7 +886,8 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <f>4-SUM(D2:G2)</f>
+        <v>0</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -885,16 +899,19 @@
         <v>1</v>
       </c>
       <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>16</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>4</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -902,7 +919,8 @@
         <v>8</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <f t="shared" ref="C3:C46" si="0">4-SUM(D3:G3)</f>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -914,16 +932,19 @@
         <v>1</v>
       </c>
       <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
         <v>15</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>5</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -931,7 +952,8 @@
         <v>11</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -943,16 +965,19 @@
         <v>1</v>
       </c>
       <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
         <v>14</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>6</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -960,7 +985,8 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -972,16 +998,19 @@
         <v>1</v>
       </c>
       <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
         <v>13</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>7</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -989,10 +1018,11 @@
         <v>17</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -1001,16 +1031,19 @@
         <v>1</v>
       </c>
       <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
         <v>12</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>8</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1018,7 +1051,8 @@
         <v>20</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1030,16 +1064,19 @@
         <v>1</v>
       </c>
       <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
         <v>11</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>9</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1047,7 +1084,8 @@
         <v>23</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1059,16 +1097,19 @@
         <v>1</v>
       </c>
       <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
         <v>10</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>16</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1076,7 +1117,8 @@
         <v>26</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1088,16 +1130,19 @@
         <v>1</v>
       </c>
       <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
         <v>9</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>11</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1105,7 +1150,8 @@
         <v>29</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1117,16 +1163,19 @@
         <v>1</v>
       </c>
       <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
         <v>8</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>12</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -1134,7 +1183,8 @@
         <v>32</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1146,16 +1196,19 @@
         <v>1</v>
       </c>
       <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
         <v>7</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>13</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1163,10 +1216,11 @@
         <v>35</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -1175,16 +1229,19 @@
         <v>1</v>
       </c>
       <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
         <v>6</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>14</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1192,7 +1249,8 @@
         <v>38</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1204,16 +1262,19 @@
         <v>1</v>
       </c>
       <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
         <v>5</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>15</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>40</v>
       </c>
@@ -1221,7 +1282,8 @@
         <v>41</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1233,16 +1295,19 @@
         <v>1</v>
       </c>
       <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
         <v>4</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>16</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -1250,7 +1315,8 @@
         <v>44</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1262,16 +1328,19 @@
         <v>1</v>
       </c>
       <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
         <v>16</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>4</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>46</v>
       </c>
@@ -1279,7 +1348,8 @@
         <v>47</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1291,16 +1361,19 @@
         <v>1</v>
       </c>
       <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
         <v>15</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>5</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -1308,28 +1381,32 @@
         <v>50</v>
       </c>
       <c r="C17">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
         <v>14</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>6</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -1337,7 +1414,8 @@
         <v>52</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1349,16 +1427,19 @@
         <v>1</v>
       </c>
       <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
         <v>13</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>7</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -1366,7 +1447,8 @@
         <v>55</v>
       </c>
       <c r="C19">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1378,16 +1460,19 @@
         <v>1</v>
       </c>
       <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
         <v>12</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>8</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>57</v>
       </c>
@@ -1395,7 +1480,8 @@
         <v>58</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1407,16 +1493,19 @@
         <v>1</v>
       </c>
       <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
         <v>11</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>9</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>60</v>
       </c>
@@ -1424,7 +1513,8 @@
         <v>61</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1436,16 +1526,19 @@
         <v>1</v>
       </c>
       <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
         <v>10</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>16</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>63</v>
       </c>
@@ -1453,7 +1546,8 @@
         <v>64</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -1465,16 +1559,19 @@
         <v>1</v>
       </c>
       <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
         <v>9</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>11</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>66</v>
       </c>
@@ -1482,7 +1579,8 @@
         <v>67</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1494,16 +1592,19 @@
         <v>1</v>
       </c>
       <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
         <v>8</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>12</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -1511,7 +1612,8 @@
         <v>70</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1523,16 +1625,19 @@
         <v>1</v>
       </c>
       <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
         <v>7</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>13</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>72</v>
       </c>
@@ -1540,7 +1645,8 @@
         <v>73</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -1552,16 +1658,19 @@
         <v>1</v>
       </c>
       <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
         <v>6</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>14</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>75</v>
       </c>
@@ -1569,7 +1678,8 @@
         <v>76</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1581,16 +1691,19 @@
         <v>1</v>
       </c>
       <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
         <v>5</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>15</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -1598,7 +1711,8 @@
         <v>79</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -1610,16 +1724,19 @@
         <v>1</v>
       </c>
       <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
         <v>4</v>
       </c>
-      <c r="H27">
+      <c r="I27">
         <v>16</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>81</v>
       </c>
@@ -1627,7 +1744,8 @@
         <v>82</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1639,16 +1757,19 @@
         <v>1</v>
       </c>
       <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28">
         <v>16</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>4</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>84</v>
       </c>
@@ -1656,7 +1777,8 @@
         <v>85</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1668,16 +1790,19 @@
         <v>1</v>
       </c>
       <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
         <v>15</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>5</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>87</v>
       </c>
@@ -1685,7 +1810,8 @@
         <v>88</v>
       </c>
       <c r="C30">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1697,16 +1823,19 @@
         <v>1</v>
       </c>
       <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
         <v>14</v>
       </c>
-      <c r="H30">
+      <c r="I30">
         <v>6</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>90</v>
       </c>
@@ -1714,7 +1843,8 @@
         <v>91</v>
       </c>
       <c r="C31">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1726,16 +1856,19 @@
         <v>1</v>
       </c>
       <c r="G31">
+        <v>1</v>
+      </c>
+      <c r="H31">
         <v>13</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>7</v>
       </c>
-      <c r="I31" t="s">
+      <c r="J31" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>93</v>
       </c>
@@ -1743,7 +1876,8 @@
         <v>94</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -1755,16 +1889,19 @@
         <v>1</v>
       </c>
       <c r="G32">
+        <v>1</v>
+      </c>
+      <c r="H32">
         <v>12</v>
       </c>
-      <c r="H32">
+      <c r="I32">
         <v>8</v>
       </c>
-      <c r="I32" t="s">
+      <c r="J32" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>96</v>
       </c>
@@ -1772,7 +1909,8 @@
         <v>97</v>
       </c>
       <c r="C33">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -1784,16 +1922,19 @@
         <v>1</v>
       </c>
       <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="H33">
         <v>11</v>
       </c>
-      <c r="H33">
+      <c r="I33">
         <v>9</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>22</v>
       </c>
@@ -1801,7 +1942,8 @@
         <v>99</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -1813,16 +1955,19 @@
         <v>1</v>
       </c>
       <c r="G34">
+        <v>1</v>
+      </c>
+      <c r="H34">
         <v>10</v>
       </c>
-      <c r="H34">
+      <c r="I34">
         <v>16</v>
       </c>
-      <c r="I34" t="s">
+      <c r="J34" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>101</v>
       </c>
@@ -1830,48 +1975,56 @@
         <v>102</v>
       </c>
       <c r="C35">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35">
         <v>1</v>
       </c>
       <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35">
         <v>9</v>
       </c>
-      <c r="H35">
+      <c r="I35">
         <v>11</v>
       </c>
-      <c r="I35" t="s">
+      <c r="J35" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>104</v>
       </c>
       <c r="B36" t="s">
         <v>105</v>
       </c>
-      <c r="D36">
-        <v>0</v>
-      </c>
-      <c r="G36">
+      <c r="C36">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="H36">
         <v>8</v>
       </c>
-      <c r="H36">
+      <c r="I36">
         <v>12</v>
       </c>
-      <c r="I36" t="s">
+      <c r="J36" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>107</v>
       </c>
@@ -1879,7 +2032,8 @@
         <v>108</v>
       </c>
       <c r="C37">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1891,16 +2045,19 @@
         <v>1</v>
       </c>
       <c r="G37">
+        <v>1</v>
+      </c>
+      <c r="H37">
         <v>7</v>
       </c>
-      <c r="H37">
+      <c r="I37">
         <v>13</v>
       </c>
-      <c r="I37" t="s">
+      <c r="J37" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>110</v>
       </c>
@@ -1908,7 +2065,8 @@
         <v>111</v>
       </c>
       <c r="C38">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -1920,16 +2078,19 @@
         <v>1</v>
       </c>
       <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38">
         <v>6</v>
       </c>
-      <c r="H38">
+      <c r="I38">
         <v>14</v>
       </c>
-      <c r="I38" t="s">
+      <c r="J38" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>113</v>
       </c>
@@ -1937,7 +2098,8 @@
         <v>114</v>
       </c>
       <c r="C39">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -1949,16 +2111,19 @@
         <v>1</v>
       </c>
       <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
         <v>5</v>
       </c>
-      <c r="H39">
+      <c r="I39">
         <v>15</v>
       </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>116</v>
       </c>
@@ -1966,10 +2131,11 @@
         <v>117</v>
       </c>
       <c r="C40">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="D40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -1978,16 +2144,19 @@
         <v>1</v>
       </c>
       <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40">
         <v>4</v>
       </c>
-      <c r="H40">
+      <c r="I40">
         <v>16</v>
       </c>
-      <c r="I40" t="s">
+      <c r="J40" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>119</v>
       </c>
@@ -1995,7 +2164,8 @@
         <v>120</v>
       </c>
       <c r="C41">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -2007,16 +2177,19 @@
         <v>1</v>
       </c>
       <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="H41">
         <v>16</v>
       </c>
-      <c r="H41">
+      <c r="I41">
         <v>4</v>
       </c>
-      <c r="I41" t="s">
+      <c r="J41" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>122</v>
       </c>
@@ -2024,6 +2197,7 @@
         <v>123</v>
       </c>
       <c r="C42">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D42">
@@ -2033,19 +2207,22 @@
         <v>1</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
         <v>15</v>
       </c>
-      <c r="H42">
+      <c r="I42">
         <v>5</v>
       </c>
-      <c r="I42" t="s">
+      <c r="J42" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>125</v>
       </c>
@@ -2053,7 +2230,8 @@
         <v>126</v>
       </c>
       <c r="C43">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -2065,16 +2243,19 @@
         <v>1</v>
       </c>
       <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="H43">
         <v>14</v>
       </c>
-      <c r="H43">
+      <c r="I43">
         <v>6</v>
       </c>
-      <c r="I43" t="s">
+      <c r="J43" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>128</v>
       </c>
@@ -2082,7 +2263,8 @@
         <v>129</v>
       </c>
       <c r="C44">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -2094,16 +2276,19 @@
         <v>1</v>
       </c>
       <c r="G44">
+        <v>1</v>
+      </c>
+      <c r="H44">
         <v>13</v>
       </c>
-      <c r="H44">
+      <c r="I44">
         <v>7</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>131</v>
       </c>
@@ -2111,7 +2296,8 @@
         <v>132</v>
       </c>
       <c r="C45">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -2123,16 +2309,19 @@
         <v>1</v>
       </c>
       <c r="G45">
+        <v>1</v>
+      </c>
+      <c r="H45">
         <v>12</v>
       </c>
-      <c r="H45">
+      <c r="I45">
         <v>8</v>
       </c>
-      <c r="I45" t="s">
+      <c r="J45" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>134</v>
       </c>
@@ -2140,24 +2329,28 @@
         <v>135</v>
       </c>
       <c r="C46">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D46">
         <v>1</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46">
         <v>11</v>
       </c>
-      <c r="H46">
+      <c r="I46">
         <v>9</v>
       </c>
-      <c r="I46" t="s">
+      <c r="J46" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>